<commit_message>
update new results data
</commit_message>
<xml_diff>
--- a/src/data/results.xlsx
+++ b/src/data/results.xlsx
@@ -11,6 +11,64 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
+  <authors>
+    <author>tc={9d7c1cdf-b27a-4c14-8172-6a42d27fd905}</author>
+    <author>tc={eef30766-c68a-4c27-ae44-90be151ace47}</author>
+  </authors>
+  <commentList>
+    <comment authorId="0" xr:uid="{9d7c1cdf-b27a-4c14-8172-6a42d27fd905}" ref="D2">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+ Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+	updated this
+</t>
+      </text>
+    </comment>
+    <comment authorId="1" xr:uid="{eef30766-c68a-4c27-ae44-90be151ace47}" ref="C2">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+ Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+	updated this
+</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
+  <authors>
+    <author>tc={10579042-d9c6-41d3-b4b1-246975e33844}</author>
+    <author>tc={67f2873d-6fc4-4c2c-94bf-7d21b48dfe3b}</author>
+  </authors>
+  <commentList>
+    <comment authorId="0" xr:uid="{10579042-d9c6-41d3-b4b1-246975e33844}" ref="C3">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+ Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+	updated this
+</t>
+      </text>
+    </comment>
+    <comment authorId="1" xr:uid="{67f2873d-6fc4-4c2c-94bf-7d21b48dfe3b}" ref="B5">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+ Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+	updated this
+</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="40">
   <si>
@@ -26,16 +84,28 @@
     <t>Description</t>
   </si>
   <si>
+    <t>Deepan Raju</t>
+  </si>
+  <si>
+    <t>BJT &amp; RLC Circuit Analyzer</t>
+  </si>
+  <si>
+    <t>It is a Scilab GUI for Electronics Engineering students to simulate RLC circuits and BJT amplifiers (CE, CB, CC). It calculates resonant frequency, gain, bandwidth, and cutoff frequencies, with frequency-response plots and lab-format observation tables</t>
+  </si>
+  <si>
+    <t>Chirag paliwal</t>
+  </si>
+  <si>
     <t>Amirtha K</t>
   </si>
   <si>
-    <t>GUIVerse - Interactive Digital Communication System Laboratory in Scilab</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Scilab-based digital communication laboratory that visualizes the complete signal-processing pipeline: analog signal generation, sampling, aliasing detection, Whittaker reconstruction, uniform/non-uniform quantization, SQNR analysis, PCM encoding, and serialized transmission</t>
-  </si>
-  <si>
-    <t>Deepan Raju</t>
+    <t>Interactive Digital Communication System Laboratory in Scilab</t>
+  </si>
+  <si>
+    <t>DTC3_Digital Twin Command Center</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> It is a digital communication laboratory that visualizes the complete signal-processing pipeline: analog signal generation, sampling, aliasing detection, Whittaker reconstruction, uniform/non-uniform quantization, SQNR analysis, PCM encoding, and serialized transmission.</t>
   </si>
   <si>
     <t>Ullas R</t>
@@ -47,46 +117,70 @@
     <t>SolarVista is an interactive Scilab GUI for rooftop solar PV planning. It estimates system capacity, panel requirements, energy generation, savings, payback period, and CO₂ reduction based on roof, location, panel, and tariff inputs. It also provides monthly generation charts and a visual panel layout for technical, financial, and environmental assessment.</t>
   </si>
   <si>
-    <t>BJT &amp; RLC Circuit Analyzer</t>
+    <t>DTC3 is a Scilab-based AI-powered Digital Twin Command Center for industrial plant monitoring. It simulates live sensor data, predicts equipment failures, visualizes component health, provides real-time analytics, and generates AI-based maintenance reports for predictive maintenance and safety.</t>
+  </si>
+  <si>
+    <t>V S Vigesh</t>
+  </si>
+  <si>
+    <t>Spring-Mass-Damper &amp; Projectile Motion</t>
+  </si>
+  <si>
+    <t>A Scilab GUI combining Spring-Mass-Damper and Projectile Motion simulators in one interactive window. Users adjust parameters with sliders and view damping behavior, range, height, time, scenario comparisons, animations, and PNG/CSV exports. It provides a hands-on physics learning experience.</t>
   </si>
   <si>
     <t>Nalinkumar S</t>
   </si>
   <si>
+    <t>Harish Kumar P S</t>
+  </si>
+  <si>
     <t>LabTwin: Interactive System Identification Studio</t>
   </si>
   <si>
+    <t>Solar Panel Performance &amp; Optimization Simulator</t>
+  </si>
+  <si>
     <t>LabTwin is a Scilab GUI that turns noisy lab CSV data into physical models. Students analyze traces using time series, FFT, and histograms, choose from four physical laws, and estimate constants using sliders or least-squares fitting. It also includes model ranking, system animation, and a Challenge Mode with mystery traces.</t>
   </si>
   <si>
-    <t>It is a Scilab GUI for Electronics Engineering students to simulate RLC circuits and BJT amplifiers (CE, CB, CC). It calculates resonant frequency, gain, bandwidth, and cutoff frequencies, with frequency-response plots and lab-format observation tables</t>
+    <t>A Scilab-based solar PV simulator that models irradiance, solar position, cell temperature, DC/AC power, system losses, and hourly energy generation. It also optimizes panel tilt and provides interactive graphs and scenario comparisons.</t>
+  </si>
+  <si>
+    <t>Lekhraj</t>
+  </si>
+  <si>
+    <t>Personal DSA Operating System</t>
+  </si>
+  <si>
+    <t>It is an offline-first Scilab GUI application for coding interview preparation. It combines DSA problem tracking, spaced revision, journaling, analytics, and report generation in one desktop workspace.</t>
   </si>
   <si>
     <t>Vaibhav Suvagiya</t>
   </si>
   <si>
-    <t>Chirag paliwal</t>
-  </si>
-  <si>
-    <t>DTC3_DIGITAL TWIN COMMAND CENTER</t>
-  </si>
-  <si>
-    <t>DTC3 is a Scilab-based AI-powered Digital Twin Command Center for industrial plant monitoring. It simulates live sensor data, predicts equipment failures, visualizes component health, provides real-time analytics, and generates AI-based maintenance reports for predictive maintenance and safety.</t>
+    <t>Ridham Dipakkumar Kevat</t>
+  </si>
+  <si>
+    <t>SciCircuits: Circuit Simulator &amp; GUI in Scilab</t>
+  </si>
+  <si>
+    <t>SciCircuits is an interactive Scilab circuit simulator with a GUI, pre-built RC, RLC, Op-Amp, and diode circuits, plus a code-based netlist parser. It uses matrix solvers for transient, AC Bode, and DC sweep analysis.</t>
   </si>
   <si>
     <t>PID Playground: Interactive Control Systems Tuning Studio</t>
   </si>
   <si>
-    <t>V S Vigesh</t>
-  </si>
-  <si>
-    <t>Spring-Mass-Damper &amp; Projectile Motion</t>
+    <t>Vian Mangal</t>
+  </si>
+  <si>
+    <t>PowerLens - Interactive Power Quality and Harmonic Simulator</t>
   </si>
   <si>
     <t>PID Playground is an interactive Scilab GUI for learning PID tuning. It includes real-world plants, Challenge Mode, individual P/I/D contributions, and CSV/PNG export.</t>
   </si>
   <si>
-    <t>A Scilab GUI combining Spring-Mass-Damper and Projectile Motion simulators in one interactive window. Users adjust parameters with sliders and view damping behavior, range, height, time, scenario comparisons, animations, and PNG/CSV exports. It provides a hands-on physics learning experience.</t>
+    <t>PowerLens is an interactive Scilab simulator for exploring harmonics, voltage sag, and interference in AC supplies. Users adjust signal parameters and compare waveforms, FFT spectrum, RMS voltage, THD, crest factor, and dominant harmonics.</t>
   </si>
   <si>
     <t>Sneha Dubey</t>
@@ -95,43 +189,7 @@
     <t>Multi-Physics Simulator Suite</t>
   </si>
   <si>
-    <t>HARISH KUMAR P S</t>
-  </si>
-  <si>
     <t>It combines eight core physics and engineering phenomena in one interactive learning platform. Users adjust parameters through sliders and dropdowns and watch the underlying science animate and solve in real time.</t>
-  </si>
-  <si>
-    <t>Solar Panel Performance &amp; Optimization Simulator</t>
-  </si>
-  <si>
-    <t>A Scilab-based solar PV simulator that models irradiance, solar position, cell temperature, DC/AC power, system losses, and hourly energy generation. It also optimizes panel tilt and provides interactive graphs and scenario comparisons.</t>
-  </si>
-  <si>
-    <t>Lekhraj</t>
-  </si>
-  <si>
-    <t>Personal DSA Operating System</t>
-  </si>
-  <si>
-    <t>Lekhraj is an offline-first Scilab GUI application for coding interview preparation. It combines DSA problem tracking, spaced revision, journaling, analytics, and report generation in one desktop workspace.</t>
-  </si>
-  <si>
-    <t>Ridham Dipakkumar Kevat</t>
-  </si>
-  <si>
-    <t>SciCircuits: Circuit Simulator &amp; GUI in Scilab</t>
-  </si>
-  <si>
-    <t>SciCircuits is an interactive Scilab circuit simulator with a GUI, pre-built RC, RLC, Op-Amp, and diode circuits, plus a code-based netlist parser. It uses matrix solvers for transient, AC Bode, and DC sweep analysis.</t>
-  </si>
-  <si>
-    <t>Vian Mangal</t>
-  </si>
-  <si>
-    <t>PowerLens - Interactive Power Quality and Harmonic Simulator</t>
-  </si>
-  <si>
-    <t>PowerLens is an interactive Scilab simulator for exploring harmonics, voltage sag, and interference in AC supplies. Users adjust signal parameters and compare waveforms, FFT spectrum, RMS voltage, THD, crest factor, and dominant harmonics.</t>
   </si>
 </sst>
 </file>
@@ -152,11 +210,6 @@
       <name val="Arial"/>
     </font>
     <font>
-      <sz val="11.0"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-    </font>
-    <font>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
@@ -167,12 +220,17 @@
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
-    <font/>
     <font>
       <sz val="11.0"/>
       <color rgb="FF000000"/>
       <name val="Inherit"/>
     </font>
+    <font>
+      <sz val="11.0"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+    </font>
+    <font/>
     <font>
       <sz val="11.0"/>
       <color theme="1"/>
@@ -242,27 +300,27 @@
     <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="2" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="2" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="2" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="3" fillId="0" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="1" fillId="2" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
+    <xf borderId="2" fillId="2" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="0" fontId="6" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="1" fillId="2" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -272,6 +330,14 @@
 </styleSheet>
 </file>
 
+<file path=xl/documenttasks/documenttask1.xml><?xml version="1.0" encoding="utf-8"?>
+<Tasks xmlns="http://schemas.microsoft.com/office/tasks/2019/documenttasks"/>
+</file>
+
+<file path=xl/documenttasks/documenttask2.xml><?xml version="1.0" encoding="utf-8"?>
+<Tasks xmlns="http://schemas.microsoft.com/office/tasks/2019/documenttasks"/>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
@@ -281,7 +347,9 @@
 </file>
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
+<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
+  <x18tc:person displayName="Scilab Team Fossee" id="{ae0a87ef-3450-4984-88be-055b1677d798}" providerId="google-sheets"/>
+</x18tc:personList>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -478,6 +546,28 @@
 </a:theme>
 </file>
 
+<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
+<x18tc:ThreadedComments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <x18tc:threadedComment ref="C2" dT="2026-09-18T07:32:09.00" personId="{ae0a87ef-3450-4984-88be-055b1677d798}" id="{eef30766-c68a-4c27-ae44-90be151ace47}" done="0">
+    <x18tc:text xml:space="preserve">updated this</x18tc:text>
+  </x18tc:threadedComment>
+  <x18tc:threadedComment ref="D2" dT="2026-09-18T07:32:56.00" personId="{ae0a87ef-3450-4984-88be-055b1677d798}" id="{9d7c1cdf-b27a-4c14-8172-6a42d27fd905}" done="0">
+    <x18tc:text xml:space="preserve">updated this</x18tc:text>
+  </x18tc:threadedComment>
+</x18tc:ThreadedComments>
+</file>
+
+<file path=xl/threadedComments/threadedComment2.xml><?xml version="1.0" encoding="utf-8"?>
+<x18tc:ThreadedComments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <x18tc:threadedComment ref="C3" dT="2026-09-18T07:36:17.00" personId="{ae0a87ef-3450-4984-88be-055b1677d798}" id="{10579042-d9c6-41d3-b4b1-246975e33844}" done="0">
+    <x18tc:text xml:space="preserve">updated this</x18tc:text>
+  </x18tc:threadedComment>
+  <x18tc:threadedComment ref="B5" dT="2026-09-18T07:33:32.00" personId="{ae0a87ef-3450-4984-88be-055b1677d798}" id="{67f2873d-6fc4-4c2c-94bf-7d21b48dfe3b}" done="0">
+    <x18tc:text xml:space="preserve">updated this</x18tc:text>
+  </x18tc:threadedComment>
+</x18tc:ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
@@ -504,69 +594,69 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2">
+      <c r="A2" s="5">
         <v>1.0</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>6</v>
+      <c r="B2" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4">
+      <c r="A3" s="7">
         <v>2.0</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>10</v>
+      <c r="B3" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6"/>
-      <c r="B4" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>14</v>
+      <c r="A4" s="8"/>
+      <c r="B4" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4">
+      <c r="A5" s="7">
         <v>3.0</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>23</v>
+      <c r="B5" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6"/>
-      <c r="B6" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>28</v>
+      <c r="A6" s="8"/>
+      <c r="B6" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>39</v>
       </c>
     </row>
   </sheetData>
@@ -574,7 +664,8 @@
     <mergeCell ref="A3:A4"/>
     <mergeCell ref="A5:A6"/>
   </mergeCells>
-  <drawing r:id="rId1"/>
+  <drawing r:id="rId4"/>
+  <legacyDrawing r:id="rId5"/>
 </worksheet>
 </file>
 
@@ -584,6 +675,10 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <cols>
+    <col customWidth="1" min="2" max="2" width="22.88"/>
+    <col customWidth="1" min="4" max="4" width="49.5"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
@@ -600,104 +695,105 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3">
+      <c r="A2" s="2">
         <v>1.0</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2">
+        <v>2.0</v>
+      </c>
+      <c r="B3" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="D2" s="5" t="s">
+      <c r="C3" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" s="3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="3">
-        <v>2.0</v>
-      </c>
-      <c r="B3" s="2" t="s">
+    <row r="4">
+      <c r="A4" s="2">
+        <v>3.0</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="D4" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D3" s="5" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3">
-        <v>3.0</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="C4" s="2" t="s">
+    </row>
+    <row r="5">
+      <c r="A5" s="2">
+        <v>4.0</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D5" s="3" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="3">
-        <v>4.0</v>
-      </c>
-      <c r="B5" s="2" t="s">
+    <row r="6">
+      <c r="A6" s="2">
+        <v>5.0</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="D6" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="C5" s="2" t="s">
+    </row>
+    <row r="7">
+      <c r="A7" s="2">
+        <v>6.0</v>
+      </c>
+      <c r="B7" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="C7" s="5" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3">
-        <v>5.0</v>
-      </c>
-      <c r="B6" s="2" t="s">
+      <c r="D7" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="C6" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="D6" s="5" t="s">
+    </row>
+    <row r="8">
+      <c r="A8" s="2">
+        <v>7.0</v>
+      </c>
+      <c r="B8" s="5" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3">
-        <v>6.0</v>
-      </c>
-      <c r="B7" s="2" t="s">
+      <c r="C8" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="C7" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D7" s="5" t="s">
+      <c r="D8" s="3" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="3">
-        <v>7.0</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>39</v>
-      </c>
-    </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <drawing r:id="rId4"/>
+  <legacyDrawing r:id="rId5"/>
 </worksheet>
 </file>
</xml_diff>